<commit_message>
logic follows TA-DM map for USUBJID-ARM
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -6,6 +6,8 @@
     <sheet name="Library" sheetId="1" r:id="rId1"/>
     <sheet name="Datasets" sheetId="2" r:id="rId2"/>
     <sheet name="ta.xpt" sheetId="3" r:id="rId3"/>
+    <sheet name="dm.xpt" sheetId="4" r:id="rId4"/>
+    <sheet name="ae.xpt" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -35,11 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -58,8 +56,23 @@
       <name val="Calibri"/>
       <i/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -67,6 +80,24 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -96,13 +127,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,18 +470,18 @@
   <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="2" t="str">
         <v>Product</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="2" t="str">
         <v>Version</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="2" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="2" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -461,69 +494,76 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="str">
+      <c r="A1" s="2" t="str">
         <v>Filename</v>
       </c>
-      <c r="B1" s="3" t="str">
+      <c r="B1" s="2" t="str">
         <v>Label</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="str">
+      <c r="A2" s="2" t="str">
         <v>ta.xpt</v>
       </c>
-      <c r="B2" s="3" t="str">
+      <c r="B2" s="2" t="str">
         <v>Trial Arms</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>Demographics</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>Adverse Events</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:G11"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="str">
+      <c r="A1" s="3" t="str">
         <v>STUDYID</v>
       </c>
-      <c r="B1" s="4" t="str">
+      <c r="B1" s="3" t="str">
         <v>DOMAIN</v>
       </c>
-      <c r="C1" s="4" t="str">
+      <c r="C1" s="3" t="str">
         <v>ARMCD</v>
       </c>
-      <c r="D1" s="4" t="str">
+      <c r="D1" s="3" t="str">
         <v>ARM</v>
       </c>
-      <c r="E1" s="4" t="str">
+      <c r="E1" s="3" t="str">
         <v>TAETORD</v>
       </c>
-      <c r="F1" s="4" t="str">
+      <c r="F1" s="3" t="str">
         <v>ETCD</v>
       </c>
-      <c r="G1" s="4" t="str">
+      <c r="G1" s="3" t="str">
         <v>ELEMENT</v>
       </c>
-      <c r="H1" s="4" t="str">
-        <v>TABRANCH</v>
-      </c>
-      <c r="I1" s="4" t="str">
-        <v>TATRANS</v>
-      </c>
-      <c r="J1" s="4" t="str">
-        <v>EPOCH</v>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="4" t="str">
         <v>Study Identifier</v>
       </c>
       <c r="B2" s="5" t="str">
@@ -532,351 +572,606 @@
       <c r="C2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Planned Order of Element within Arm</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Element Code</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Description of Element</v>
       </c>
-      <c r="H2" s="5" t="str">
-        <v>Branch</v>
-      </c>
-      <c r="I2" s="5" t="str">
-        <v>Transition Rule</v>
-      </c>
-      <c r="J2" s="5" t="str">
-        <v>Epoch</v>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
+      <c r="A3" s="4" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="str">
+      <c r="A4" s="7">
         <v>12</v>
       </c>
-      <c r="B4" s="5" t="str">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="str">
+      <c r="C4" s="6">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6">
+        <v>40</v>
+      </c>
+      <c r="E4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5" t="str">
-        <v>28</v>
-      </c>
-      <c r="E4" s="5" t="str">
+      <c r="F4" s="6">
         <v>8</v>
       </c>
-      <c r="F4" s="5" t="str">
-        <v>7</v>
-      </c>
-      <c r="G4" s="5" t="str">
-        <v>26</v>
-      </c>
-      <c r="H4" s="5" t="str">
-        <v>200</v>
-      </c>
-      <c r="I4" s="5" t="str">
-        <v>200</v>
-      </c>
-      <c r="J4" s="5" t="str">
-        <v>9</v>
+      <c r="G4" s="6">
+        <v>40</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="3" t="str">
+      <c r="A5" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B5" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C5" s="3" t="str">
-        <v>PLACEBO</v>
-      </c>
-      <c r="D5" s="3" t="str">
-        <v>Placebo</v>
-      </c>
-      <c r="E5" s="3" t="str">
+      <c r="C5" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>Drug A</v>
+      </c>
+      <c r="E5" s="2">
         <v>1</v>
       </c>
-      <c r="F5" s="3" t="str">
-        <v>SCREEN</v>
-      </c>
-      <c r="G5" s="3" t="str">
-        <v>Screening</v>
-      </c>
-      <c r="H5" s="3" t="str">
-        <v>Randomized to Placebo</v>
-      </c>
-      <c r="I5" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J5" s="3" t="str">
-        <v>SCREENING</v>
+      <c r="F5" s="2" t="str">
+        <v>EL1</v>
+      </c>
+      <c r="G5" s="2" t="str">
+        <v>Element 1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="3" t="str">
+      <c r="A6" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B6" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C6" s="3" t="str">
-        <v>PLACEBO</v>
-      </c>
-      <c r="D6" s="3" t="str">
-        <v>Placebo</v>
-      </c>
-      <c r="E6" s="3" t="str">
+      <c r="C6" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>Drug A</v>
+      </c>
+      <c r="E6" s="2">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="str">
-        <v>PLACEBO</v>
-      </c>
-      <c r="G6" s="3" t="str">
-        <v>Placebo</v>
-      </c>
-      <c r="H6" s="3" t="str">
-        <v/>
-      </c>
-      <c r="I6" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J6" s="3" t="str">
-        <v>TREATMENT</v>
+      <c r="F6" s="2" t="str">
+        <v>EL2</v>
+      </c>
+      <c r="G6" s="2" t="str">
+        <v>Element 2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B7" s="3" t="str">
+      <c r="A7" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B7" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C7" s="3" t="str">
-        <v>ZAN_LOW</v>
-      </c>
-      <c r="D7" s="3" t="str">
-        <v>Zanomaline Low Dose (54 mg)</v>
-      </c>
-      <c r="E7" s="3" t="str">
+      <c r="C7" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>Drug A</v>
+      </c>
+      <c r="E7" s="2">
+        <v>3</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>EL3</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <v>Element 3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>TA</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>Drug B</v>
+      </c>
+      <c r="E8" s="2">
         <v>1</v>
       </c>
-      <c r="F7" s="3" t="str">
-        <v>SCREEN</v>
-      </c>
-      <c r="G7" s="3" t="str">
-        <v>Screening</v>
-      </c>
-      <c r="H7" s="3" t="str">
-        <v>Randomized to Zanomaline Low Dose</v>
-      </c>
-      <c r="I7" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J7" s="3" t="str">
-        <v>SCREENING</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="3" t="str">
+      <c r="F8" s="2" t="str">
+        <v>EL1</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v>Element 1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B9" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C8" s="3" t="str">
-        <v>ZAN_LOW</v>
-      </c>
-      <c r="D8" s="3" t="str">
-        <v>Zanomaline Low Dose (54 mg)</v>
-      </c>
-      <c r="E8" s="3" t="str">
+      <c r="C9" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="D9" s="2" t="str">
+        <v>Drug B</v>
+      </c>
+      <c r="E9" s="2">
         <v>2</v>
       </c>
-      <c r="F8" s="3" t="str">
-        <v>LOW</v>
-      </c>
-      <c r="G8" s="3" t="str">
-        <v>Zanomaline 54 mg</v>
-      </c>
-      <c r="H8" s="3" t="str">
-        <v/>
-      </c>
-      <c r="I8" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J8" s="3" t="str">
-        <v>TREATMENT</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B9" s="3" t="str">
+      <c r="F9" s="2" t="str">
+        <v>EL2</v>
+      </c>
+      <c r="G9" s="2" t="str">
+        <v>Element 2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B10" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C9" s="3" t="str">
-        <v>ZAN_HIGH</v>
-      </c>
-      <c r="D9" s="3" t="str">
-        <v>Zanomaline High Dose (81 mg)</v>
-      </c>
-      <c r="E9" s="3" t="str">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="str">
-        <v>SCREEN</v>
-      </c>
-      <c r="G9" s="3" t="str">
-        <v>Screening</v>
-      </c>
-      <c r="H9" s="3" t="str">
-        <v>Randomized to Zanomaline High Dose</v>
-      </c>
-      <c r="I9" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J9" s="3" t="str">
-        <v>SCREENING</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="3" t="str">
+      <c r="C10" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="D10" s="2" t="str">
+        <v>Drug B</v>
+      </c>
+      <c r="E10" s="2">
+        <v>3</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>EL3</v>
+      </c>
+      <c r="G10" s="2" t="str">
+        <v>Element 3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B11" s="2" t="str">
         <v>TA</v>
       </c>
-      <c r="C10" s="3" t="str">
-        <v>ZAN_HIGH</v>
-      </c>
-      <c r="D10" s="3" t="str">
-        <v>Zanomaline High Dose (81 mg)</v>
-      </c>
-      <c r="E10" s="3">
-        <v>2</v>
-      </c>
-      <c r="F10" s="3" t="str">
-        <v>TITRATE</v>
-      </c>
-      <c r="G10" s="3" t="str">
-        <v>Zanomaline 54 mg Titration</v>
-      </c>
-      <c r="H10" s="3" t="str">
-        <v/>
-      </c>
-      <c r="I10" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J10" s="3" t="str">
-        <v>TREATMENT</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B11" s="3" t="str">
-        <v>TA</v>
-      </c>
-      <c r="C11" s="3" t="str">
-        <v>ZAN_HIGH</v>
-      </c>
-      <c r="D11" s="3" t="str">
-        <v>Zanomaline High Dose (81 mg)</v>
-      </c>
-      <c r="E11" s="3">
-        <v>3</v>
-      </c>
-      <c r="F11" s="3" t="str">
-        <v>HIGH</v>
-      </c>
-      <c r="G11" s="3" t="str">
-        <v>Zanomaline 81 mg</v>
-      </c>
-      <c r="H11" s="3" t="str">
-        <v/>
-      </c>
-      <c r="I11" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J11" s="3" t="str">
-        <v>TREATMENT</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B12" s="3" t="str">
-        <v>TA</v>
-      </c>
-      <c r="C12" s="3" t="str">
-        <v>ZAN_HIGH</v>
-      </c>
-      <c r="D12" s="3" t="str">
-        <v>Zanomaline High Dose (81 mg)</v>
-      </c>
-      <c r="E12" s="3" t="str">
+      <c r="C11" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="D11" s="2" t="str">
+        <v>Drug B</v>
+      </c>
+      <c r="E11" s="2">
         <v>4</v>
       </c>
-      <c r="F12" s="3" t="str">
-        <v>TITRATE</v>
-      </c>
-      <c r="G12" s="3" t="str">
-        <v>Zanomaline 54 mg Titration</v>
-      </c>
-      <c r="H12" s="3" t="str">
-        <v/>
-      </c>
-      <c r="I12" s="3" t="str">
-        <v/>
-      </c>
-      <c r="J12" s="3" t="str">
-        <v>TREATMENT</v>
+      <c r="F11" s="2" t="str">
+        <v>EL4</v>
+      </c>
+      <c r="G11" s="2" t="str">
+        <v>Element 4</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
+        <v>STUDYID</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>DOMAIN</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>USUBJID</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>ARMCD</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>ARM</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="str">
+        <v>Study Identifier</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v>Domain Abbreviation</v>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v>Unique Subject Identifier</v>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v>Planned Arm Code</v>
+      </c>
+      <c r="E2" s="6" t="str">
+        <v>Description of Planned Arm</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6">
+        <v>12</v>
+      </c>
+      <c r="B4" s="6">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6">
+        <v>8</v>
+      </c>
+      <c r="D4" s="6">
+        <v>20</v>
+      </c>
+      <c r="E4" s="6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>DM</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>SUBJ001</v>
+      </c>
+      <c r="D5" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>Drug A</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>DM</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>SUBJ002</v>
+      </c>
+      <c r="D6" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>Drug B</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G11"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
+        <v>STUDYID</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>DOMAIN</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>USUBJID</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>AESEQ</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>AETERM</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>TAETORD</v>
+      </c>
+      <c r="G1" s="3" t="str">
+        <v>AESTDTC</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="str">
+        <v>Study Identifier</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <v>Domain Abbreviation</v>
+      </c>
+      <c r="C2" s="6" t="str">
+        <v>Unique Subject Identifier</v>
+      </c>
+      <c r="D2" s="6" t="str">
+        <v>Sequence Number</v>
+      </c>
+      <c r="E2" s="6" t="str">
+        <v>Reported Term for the Adverse Event</v>
+      </c>
+      <c r="F2" s="6" t="str">
+        <v>Planned Order of Element within Arm</v>
+      </c>
+      <c r="G2" s="6" t="str">
+        <v>Start Date/Time of Adverse Event</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Num</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6">
+        <v>12</v>
+      </c>
+      <c r="B4" s="6">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6">
+        <v>8</v>
+      </c>
+      <c r="D4" s="6">
+        <v>8</v>
+      </c>
+      <c r="E4" s="6">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6">
+        <v>8</v>
+      </c>
+      <c r="G4" s="6">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>SUBJ001</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>EVENT 1</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="str">
+        <v>2020-01-01</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <v>SUBJ001</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="str">
+        <v>EVENT 2</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2" t="str">
+        <v>2020-01-02</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>SUBJ001</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>EVENT 3</v>
+      </c>
+      <c r="F7" s="2">
+        <v>3</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <v>2020-01-03</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>SUBJ002</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>EVENT 4</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v>2020-01-01</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <v>SUBJ002</v>
+      </c>
+      <c r="D9" s="2">
+        <v>5</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>EVENT 5</v>
+      </c>
+      <c r="F9" s="2">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2" t="str">
+        <v>2020-01-02</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v>SUBJ002</v>
+      </c>
+      <c r="D10" s="2">
+        <v>6</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>EVENT 6</v>
+      </c>
+      <c r="F10" s="2">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2" t="str">
+        <v>2020-01-03</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>STUDY01</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>AE</v>
+      </c>
+      <c r="C11" s="2" t="str">
+        <v>SUBJ002</v>
+      </c>
+      <c r="D11" s="2">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>EVENT 7</v>
+      </c>
+      <c r="F11" s="2">
+        <v>4</v>
+      </c>
+      <c r="G11" s="2" t="str">
+        <v>2020-01-04</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CG0011 create: part B rule logic updated with new operator for interval
</commit_message>
<xml_diff>
--- a/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
+++ b/rules/NEW-RULE/positive/01/data/new-rule-positive-01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\NEW-RULE\positive\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9BA61A8-0ACB-4786-9F94-DCE3F0092205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F142E9E4-1E21-405D-94EA-728DA567B09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="71">
   <si>
     <t>Product</t>
   </si>
@@ -235,28 +235,19 @@
     <t>PHQ01-Poor Appetite or Overeating</t>
   </si>
   <si>
-    <t>PHQ0106</t>
-  </si>
-  <si>
-    <t>PHQ01-Feeling Bad About Yourself</t>
-  </si>
-  <si>
     <t>-P2M</t>
   </si>
   <si>
     <t>2013-12-15T10:00/2013-12-15T20:00</t>
   </si>
   <si>
-    <t>2013-12-15T10:00/-P2D</t>
-  </si>
-  <si>
     <t>P2W/2013-12-15T10:00</t>
   </si>
   <si>
-    <t>-P2D/P4W</t>
-  </si>
-  <si>
     <t>P2W</t>
+  </si>
+  <si>
+    <t>2013-12-15T10:00/P2D</t>
   </si>
 </sst>
 </file>
@@ -312,13 +303,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,7 +663,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A813908C-6C40-4ECC-9360-E46477389083}">
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="17" max="17" width="32.5703125" bestFit="1" customWidth="1"/>
@@ -941,7 +931,7 @@
         <v>1</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -994,7 +984,7 @@
         <v>1</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -1046,8 +1036,8 @@
       <c r="P7" s="3">
         <v>1</v>
       </c>
-      <c r="Q7" s="5" t="s">
-        <v>69</v>
+      <c r="Q7" s="3" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -1099,7 +1089,7 @@
       <c r="P8" s="3">
         <v>1</v>
       </c>
-      <c r="Q8" s="5" t="s">
+      <c r="Q8" s="3" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1152,61 +1142,8 @@
       <c r="P9" s="3">
         <v>1</v>
       </c>
-      <c r="Q9" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="3">
-        <v>6</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="J10" s="3">
-        <v>1</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="L10" s="3">
-        <v>3</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="P10" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q10" s="4" t="s">
-        <v>72</v>
+      <c r="Q9" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>